<commit_message>
Updated .gitignore to include TestingFiles folder and added CHANGELOG_2026-03-04.txt
</commit_message>
<xml_diff>
--- a/ClioCustomField_TestValidation.xlsx
+++ b/ClioCustomField_TestValidation.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="243" documentId="8_{3120D6FD-25C6-47F0-8A39-89B25F99CA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{147647F2-0C21-4C19-9471-946F6F5FC364}"/>
+  <xr:revisionPtr revIDLastSave="435" documentId="8_{3120D6FD-25C6-47F0-8A39-89B25F99CA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66F6C6D9-FDC2-4CD5-90DC-57695DB875FA}"/>
   <bookViews>
-    <workbookView xWindow="28665" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{DF2C5E22-660C-4BCB-A765-9F1A84EF46AA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DF2C5E22-660C-4BCB-A765-9F1A84EF46AA}"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Scenarios Clio" sheetId="1" r:id="rId1"/>
-    <sheet name="Templates" sheetId="2" r:id="rId2"/>
+    <sheet name="FunctionalTestScenarios" sheetId="1" r:id="rId1"/>
+    <sheet name="EdgeTestingScenarios" sheetId="3" r:id="rId2"/>
+    <sheet name="Templates" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="59">
   <si>
     <t>TempCode</t>
   </si>
@@ -115,13 +116,151 @@
   </si>
   <si>
     <t>Changed CF in Doc to Uppercase to see if it gets flagged this time</t>
+  </si>
+  <si>
+    <t>Fields inside tables / headers / footers</t>
+  </si>
+  <si>
+    <t>Fields that do not exist in lookup table</t>
+  </si>
+  <si>
+    <t>Duplicate old values mapped to different new values</t>
+  </si>
+  <si>
+    <r>
+      <t>Non‑docx file in folder</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> (ensure skip or fail gracefully)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Zero‑byte or corrupted docx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> in upload folder</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Large file set (700+)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> to validate stability and rate‑limit handling</t>
+    </r>
+  </si>
+  <si>
+    <t>&lt;&lt;   MATTER.CUSTOMFIELD.PLAINTIFFSNAMESHORT &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.PlaintiffsFullLegalName   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.ResponsibleAttorney   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CaseNumber&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.DefendantsFullLegalName &gt;&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;&lt;Matter.CustomField.Judge&gt;&gt; </t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.County &gt;&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inside THF Custom Field 1 - Tables (CF in Table, But Also in Paragraph) </t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OcStreetAddress &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OcCityStateZip &gt;&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inside THF Custom Field 2 - Headers (CF in Header, But Also in Paragraph) </t>
+  </si>
+  <si>
+    <t>Inside THF Custom Field 3 - Footers (CF Only in Footer)</t>
+  </si>
+  <si>
+    <t>Custom Fields for Testing</t>
+  </si>
+  <si>
+    <t>Testing Scenario/Protocol</t>
+  </si>
+  <si>
+    <t>Mixed case / spacing in custom fields (&lt;&lt; MATTER... &gt;&gt; vs &lt;&lt; Matter... &gt;&gt;)</t>
+  </si>
+  <si>
+    <t>MCS Custom Field 5 - No Spaces on Beg. of CF (3 CFs Within Template)</t>
+  </si>
+  <si>
+    <t>MCS Custom Field 6 - No Spaces on Both Beg. And End of CF (3 CFs Within Template)</t>
+  </si>
+  <si>
+    <t>MCS Custom Field 4 - No Spaces on End of CF (3 CFs Within Template)</t>
+  </si>
+  <si>
+    <t>MCS Custom Field 3 - 3 Spaces on Both Beg. and End of CF (3 CFs Within Template)</t>
+  </si>
+  <si>
+    <t>MCS Custom Field 2 - 3 Spaces on Beginning of CF (split between pages,  7 CFs Within Template)</t>
+  </si>
+  <si>
+    <t>MCS Custom Field 1 - 3 Spaces on End of CF (split between lines, 14 CFs Within Template)</t>
+  </si>
+  <si>
+    <t>&lt;&lt; TheField.ThatDoesNot.Exist &gt;&gt;</t>
+  </si>
+  <si>
+    <t>Copy Excel Doc From Testing Folder into Upload Folder</t>
+  </si>
+  <si>
+    <t>Copy Blank Word Document into Upload Folder</t>
+  </si>
+  <si>
+    <t>??</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>Notes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="171" formatCode="."/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,6 +281,20 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="12">
@@ -212,7 +365,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -343,11 +496,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -380,21 +544,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -407,8 +560,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -430,16 +582,38 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -487,6 +661,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -814,105 +992,105 @@
     <col min="3" max="3" width="57.7109375" customWidth="1"/>
     <col min="4" max="4" width="13.140625" customWidth="1"/>
     <col min="5" max="5" width="69.42578125" customWidth="1"/>
-    <col min="6" max="6" width="23.42578125" style="18" customWidth="1"/>
+    <col min="6" max="6" width="23.42578125" style="17" customWidth="1"/>
     <col min="7" max="7" width="59.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="26" t="s">
         <v>15</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="D1" s="27" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="34" t="s">
+      <c r="F1" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="32" t="s">
+      <c r="G1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="35" t="s">
+      <c r="H1" s="29" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="25"/>
-      <c r="B2" s="26" t="s">
+      <c r="A2" s="20"/>
+      <c r="B2" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="36" t="s">
+      <c r="C2" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="25">
+      <c r="D2" s="20">
         <v>2</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="25"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="30"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="25"/>
-      <c r="B3" s="26"/>
-      <c r="C3" s="37" t="s">
+      <c r="A3" s="20"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="20">
         <v>4</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="E3" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="25"/>
-      <c r="G3" s="40" t="s">
+      <c r="F3" s="20"/>
+      <c r="G3" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="30"/>
+      <c r="H3" s="24"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="25"/>
-      <c r="B4" s="26"/>
-      <c r="C4" s="38" t="s">
+      <c r="A4" s="20"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="20">
         <v>1</v>
       </c>
       <c r="E4" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="25"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="30"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="24"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="25"/>
-      <c r="B5" s="26"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="25"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="20"/>
       <c r="E5" s="11"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="30"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="24"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="36" t="s">
+      <c r="C6" s="30" t="s">
         <v>19</v>
       </c>
       <c r="D6" s="1">
@@ -928,13 +1106,13 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="11"/>
-      <c r="C7" s="37" t="s">
+      <c r="C7" s="31" t="s">
         <v>17</v>
       </c>
       <c r="D7" s="1">
         <v>4</v>
       </c>
-      <c r="E7" s="27" t="s">
+      <c r="E7" s="22" t="s">
         <v>22</v>
       </c>
       <c r="F7" s="1"/>
@@ -944,7 +1122,7 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="11"/>
-      <c r="C8" s="38" t="s">
+      <c r="C8" s="32" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="1">
@@ -960,25 +1138,25 @@
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="11"/>
-      <c r="C9" s="39"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="26"/>
+      <c r="E9" s="21"/>
       <c r="F9" s="1"/>
       <c r="G9" s="2"/>
       <c r="H9" s="10"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="21"/>
+      <c r="A10" s="1"/>
       <c r="B10" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="31" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="1">
         <v>6</v>
       </c>
-      <c r="E10" s="27" t="s">
+      <c r="E10" s="22" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="1"/>
@@ -986,9 +1164,9 @@
       <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
+      <c r="A11" s="1"/>
       <c r="B11" s="11"/>
-      <c r="C11" s="38" t="s">
+      <c r="C11" s="32" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="1">
@@ -997,58 +1175,311 @@
       <c r="E11" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="23"/>
+      <c r="F11" s="18"/>
       <c r="G11" s="3"/>
       <c r="H11" s="14"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="21"/>
+      <c r="A12" s="1"/>
       <c r="B12" s="11"/>
-      <c r="C12" s="19"/>
+      <c r="C12" s="11"/>
       <c r="D12" s="1"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="23"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="18"/>
       <c r="G12" s="3"/>
       <c r="H12" s="14"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="21"/>
+      <c r="A13" s="1"/>
       <c r="B13" s="11"/>
-      <c r="C13" s="19"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="1"/>
       <c r="E13" s="11"/>
-      <c r="F13" s="23"/>
+      <c r="F13" s="18"/>
       <c r="G13" s="3"/>
       <c r="H13" s="14"/>
     </row>
     <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="12"/>
-      <c r="C14" s="20"/>
+      <c r="C14" s="12"/>
       <c r="D14" s="4"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="24"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="5"/>
       <c r="H14" s="15"/>
     </row>
     <row r="22" spans="5:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E22" s="17"/>
+      <c r="E22" s="16"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E3">
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E3">
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F86F2E04-EE71-4EEA-BC46-ACCE4253F69D}">
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="76.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="39.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="37"/>
+      <c r="B1" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="38" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="36">
+        <v>1</v>
+      </c>
+      <c r="B2" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="36"/>
+      <c r="B3" s="43" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+    </row>
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="36"/>
+      <c r="B4" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="36"/>
+      <c r="B5" s="43" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="36"/>
+      <c r="B6" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="36"/>
+      <c r="B7" s="43" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+    </row>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="36"/>
+      <c r="B8" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="36"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="34">
+        <v>2</v>
+      </c>
+      <c r="B10" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="34"/>
+      <c r="B11" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="34"/>
+      <c r="B12" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="34"/>
+      <c r="B13" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="34"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="36">
+        <v>3</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="36">
+        <v>4</v>
+      </c>
+      <c r="B16" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="36">
+        <v>5</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="36"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="36">
+        <v>6</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="36">
+        <v>7</v>
+      </c>
+      <c r="B20" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1C990D1-0B88-44F6-819D-B6728E0DB287}">
   <dimension ref="A1:B30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Updated .gitignore to include Testing_Files folder and completed testing scripts for Custom Field Validation within the ClioCustomField_TestValidation.xlsx file..xlsx file.
</commit_message>
<xml_diff>
--- a/ClioCustomField_TestValidation.xlsx
+++ b/ClioCustomField_TestValidation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="435" documentId="8_{3120D6FD-25C6-47F0-8A39-89B25F99CA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66F6C6D9-FDC2-4CD5-90DC-57695DB875FA}"/>
+  <xr:revisionPtr revIDLastSave="685" documentId="8_{3120D6FD-25C6-47F0-8A39-89B25F99CA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A49D39BA-B205-48D6-87FC-457AC8C78DB6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DF2C5E22-660C-4BCB-A765-9F1A84EF46AA}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="82">
   <si>
     <t>TempCode</t>
   </si>
@@ -116,9 +116,6 @@
   </si>
   <si>
     <t>Changed CF in Doc to Uppercase to see if it gets flagged this time</t>
-  </si>
-  <si>
-    <t>Fields inside tables / headers / footers</t>
   </si>
   <si>
     <t>Fields that do not exist in lookup table</t>
@@ -193,48 +190,15 @@
     <t>&lt;&lt; Matter.CustomField.County &gt;&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Inside THF Custom Field 1 - Tables (CF in Table, But Also in Paragraph) </t>
-  </si>
-  <si>
     <t>&lt;&lt; Matter.CustomField.OcStreetAddress &gt;&gt;</t>
   </si>
   <si>
     <t>&lt;&lt; Matter.CustomField.OcCityStateZip &gt;&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Inside THF Custom Field 2 - Headers (CF in Header, But Also in Paragraph) </t>
-  </si>
-  <si>
-    <t>Inside THF Custom Field 3 - Footers (CF Only in Footer)</t>
-  </si>
-  <si>
-    <t>Custom Fields for Testing</t>
-  </si>
-  <si>
     <t>Testing Scenario/Protocol</t>
   </si>
   <si>
-    <t>Mixed case / spacing in custom fields (&lt;&lt; MATTER... &gt;&gt; vs &lt;&lt; Matter... &gt;&gt;)</t>
-  </si>
-  <si>
-    <t>MCS Custom Field 5 - No Spaces on Beg. of CF (3 CFs Within Template)</t>
-  </si>
-  <si>
-    <t>MCS Custom Field 6 - No Spaces on Both Beg. And End of CF (3 CFs Within Template)</t>
-  </si>
-  <si>
-    <t>MCS Custom Field 4 - No Spaces on End of CF (3 CFs Within Template)</t>
-  </si>
-  <si>
-    <t>MCS Custom Field 3 - 3 Spaces on Both Beg. and End of CF (3 CFs Within Template)</t>
-  </si>
-  <si>
-    <t>MCS Custom Field 2 - 3 Spaces on Beginning of CF (split between pages,  7 CFs Within Template)</t>
-  </si>
-  <si>
-    <t>MCS Custom Field 1 - 3 Spaces on End of CF (split between lines, 14 CFs Within Template)</t>
-  </si>
-  <si>
     <t>&lt;&lt; TheField.ThatDoesNot.Exist &gt;&gt;</t>
   </si>
   <si>
@@ -247,10 +211,295 @@
     <t>??</t>
   </si>
   <si>
-    <t>Results</t>
-  </si>
-  <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: 3 Spaces on End of CF (split between lines, 14 CFs Within Template)</t>
+    </r>
+  </si>
+  <si>
+    <t>MCS Custom Field 2: 3 Spaces on Beginning of CF (split between pages,  7 CFs Within Template)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">MCS Custom Field 3: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3 Spaces on Both Beg. and End of CF (3 CFs Within Template)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 4:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No Spaces on End of CF (3 CFs Within Template)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 5:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> No Spaces on Beg. of CF (3 CFs Within Template)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 6:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> No Spaces on Both Beg. And End of CF (3 CFs Within Template)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Inside THF Custom Field 1:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Tables (CF in Table, But Also in Paragraph) </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Inside THF Custom Field 2:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Headers (CF in Header, But Also in Paragraph) </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Inside THF Custom Field 3: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Footers (CF Only in Footer)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 7:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> CF in Uppercase in Template, While Lowercase in Lookuptable</t>
+    </r>
+  </si>
+  <si>
+    <t>Templates</t>
+  </si>
+  <si>
+    <t>ExcelDocument_4NonDocxFile_UploadFolder.xlsx</t>
+  </si>
+  <si>
+    <t>Template_UpperLowerCaseTestingScenario.docx</t>
+  </si>
+  <si>
+    <t>TemplateTesting_MixedCase_Spacing_SplitLines_Scenarios.docx</t>
+  </si>
+  <si>
+    <t>TemplateTesting_TableHeaderFooter_Scenario.docx</t>
+  </si>
+  <si>
+    <t>ZeroByteBlankDoc_UploadFolder.docx</t>
+  </si>
+  <si>
+    <t>Expected Results</t>
+  </si>
+  <si>
+    <t>Actual Results</t>
+  </si>
+  <si>
+    <t>Fields Inside Tables / Headers / Footers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Templates with Abnormal Data Structures </t>
+  </si>
+  <si>
+    <t>Additional Testing Scenarios</t>
+  </si>
+  <si>
+    <t>Mixed Case / Spacing in Custom Fields - Postive Testing</t>
+  </si>
+  <si>
+    <t>Mixed Case / Spacing in Custom Fields - Negative Testing</t>
+  </si>
+  <si>
+    <t>Custom Fields in Templates</t>
+  </si>
+  <si>
+    <t>Custom Fields in Lookup Tables</t>
+  </si>
+  <si>
+    <t>Uppercase/Lower Case Testing Scenario does not follow the Positive/Negative Testing Basis</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CaseNumber &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DefendantsFullLegalName &gt;&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;&lt; Matter.CustomField.Judge &gt;&gt; </t>
+  </si>
+  <si>
+    <t>No Custom Field</t>
+  </si>
+  <si>
+    <t>Incorrect File Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zero Bytes File </t>
+  </si>
+  <si>
+    <t>Custom Fields are Updated Successfully with all the same spaces within the Custom Field Itself</t>
+  </si>
+  <si>
+    <t>Custom Fields are NOT Updated Successfully becaue the spaces within the CF within the Templates do not Match the CFs in Lookup Table</t>
+  </si>
+  <si>
+    <t>Custom Fields are Successfully Updated within each testing scenarios table, headers, and footers CF location</t>
+  </si>
+  <si>
+    <t>&lt;&lt; MATTER.RESPONSIBLEATTORNEY.EMAIL &gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -258,9 +507,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="171" formatCode="."/>
+    <numFmt numFmtId="164" formatCode="."/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -290,14 +539,29 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -364,8 +628,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -507,11 +795,129 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -590,30 +996,124 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="171" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="14" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="14" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="14" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="14" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -652,6 +1152,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFF99"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1228,251 +1733,557 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F86F2E04-EE71-4EEA-BC46-ACCE4253F69D}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="76.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="5" width="39.85546875" customWidth="1"/>
+    <col min="2" max="2" width="88.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.42578125" style="40" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.42578125" style="40" customWidth="1"/>
+    <col min="5" max="5" width="58.85546875" style="40" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="48.5703125" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
+    <col min="8" max="8" width="39.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37"/>
-      <c r="B1" s="38" t="s">
+    <row r="1" spans="1:8" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="57"/>
+      <c r="B1" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="38" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="61"/>
+      <c r="B2" s="54" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="56"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="62"/>
+      <c r="B3" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="77" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="67"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="33"/>
+    </row>
+    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="62"/>
+      <c r="B4" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="77" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" s="68"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="33"/>
+    </row>
+    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="62"/>
+      <c r="B5" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="77" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="68"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="33"/>
+    </row>
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="62">
+        <v>1</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="77" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="70" t="s">
+        <v>78</v>
+      </c>
+      <c r="G6" s="65"/>
+      <c r="H6" s="33"/>
+    </row>
+    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="62"/>
+      <c r="B7" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="77" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="68"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="33"/>
+    </row>
+    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="62"/>
+      <c r="B8" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="77" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" s="68"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="33"/>
+    </row>
+    <row r="9" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="62"/>
+      <c r="B9" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="E9" s="77" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="69"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="33"/>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="63"/>
+      <c r="B10" s="44"/>
+      <c r="C10" s="78"/>
+      <c r="D10" s="78"/>
+      <c r="E10" s="78"/>
+      <c r="F10" s="50"/>
+      <c r="G10" s="50"/>
+      <c r="H10" s="50"/>
+    </row>
+    <row r="11" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="61"/>
+      <c r="B11" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="76"/>
+      <c r="D11" s="76"/>
+      <c r="E11" s="76"/>
+      <c r="F11" s="55"/>
+      <c r="G11" s="55"/>
+      <c r="H11" s="56"/>
+    </row>
+    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="62"/>
+      <c r="B12" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" s="67"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+    </row>
+    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="62"/>
+      <c r="B13" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" s="68"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="33"/>
+    </row>
+    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="62"/>
+      <c r="B14" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="F14" s="68"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+    </row>
+    <row r="15" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="62">
+        <v>2</v>
+      </c>
+      <c r="B15" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E15" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="F15" s="70" t="s">
+        <v>79</v>
+      </c>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+    </row>
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="62"/>
+      <c r="B16" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" s="68"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+    </row>
+    <row r="17" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="62"/>
+      <c r="B17" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="E17" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" s="68"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+    </row>
+    <row r="18" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="63"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="78"/>
+      <c r="D18" s="78"/>
+      <c r="E18" s="78"/>
+      <c r="F18" s="71"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="50"/>
+    </row>
+    <row r="19" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="61"/>
+      <c r="B19" s="54" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="76"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="76"/>
+      <c r="F19" s="66"/>
+      <c r="G19" s="55"/>
+      <c r="H19" s="56"/>
+    </row>
+    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="62"/>
+      <c r="B20" s="48" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="77" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" s="73"/>
+      <c r="G20" s="72"/>
+      <c r="H20" s="22"/>
+    </row>
+    <row r="21" spans="1:8" s="40" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A21" s="58">
+        <v>3</v>
+      </c>
+      <c r="B21" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="75" t="s">
+        <v>60</v>
+      </c>
+      <c r="F21" s="70" t="s">
+        <v>80</v>
+      </c>
+      <c r="G21" s="10"/>
+      <c r="H21" s="1"/>
+    </row>
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="62"/>
+      <c r="B22" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="75" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" s="74"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="3"/>
+    </row>
+    <row r="23" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="63"/>
+      <c r="B23" s="47"/>
+      <c r="C23" s="79"/>
+      <c r="D23" s="79"/>
+      <c r="E23" s="79"/>
+      <c r="F23" s="50"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+    </row>
+    <row r="24" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="61"/>
+      <c r="B24" s="54" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="76"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="55"/>
+      <c r="G24" s="55"/>
+      <c r="H24" s="56"/>
+    </row>
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="62"/>
+      <c r="B25" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="E25" s="20"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+    </row>
+    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="62">
+        <v>4</v>
+      </c>
+      <c r="B26" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+    </row>
+    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="62"/>
+      <c r="B27" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+    </row>
+    <row r="28" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="63"/>
+      <c r="B28" s="41"/>
+      <c r="C28" s="79"/>
+      <c r="D28" s="79"/>
+      <c r="E28" s="79"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="46"/>
+    </row>
+    <row r="29" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="64"/>
+      <c r="B29" s="54" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="76"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="76"/>
+      <c r="F29" s="55"/>
+      <c r="G29" s="55"/>
+      <c r="H29" s="56"/>
+    </row>
+    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="62"/>
+      <c r="B30" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="38" t="s">
-        <v>57</v>
-      </c>
-      <c r="E1" s="38" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="36">
-        <v>1</v>
-      </c>
-      <c r="B2" s="39" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-    </row>
-    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="36"/>
-      <c r="B3" s="43" t="s">
-        <v>52</v>
-      </c>
-      <c r="C3" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-    </row>
-    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="36"/>
-      <c r="B4" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" s="33" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="36"/>
-      <c r="B5" s="43" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" s="33" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="36"/>
-      <c r="B6" s="43" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="36"/>
-      <c r="B7" s="43" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-    </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="36"/>
-      <c r="B8" s="43" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="33" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="36"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="34">
-        <v>2</v>
-      </c>
-      <c r="B10" s="41" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="34"/>
-      <c r="B11" s="42" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="34"/>
-      <c r="B12" s="42" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="34"/>
-      <c r="B13" s="42" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="34"/>
-      <c r="B14" s="42"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="36">
-        <v>3</v>
-      </c>
-      <c r="B15" s="35" t="s">
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+    </row>
+    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="62">
+        <v>5</v>
+      </c>
+      <c r="B31" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="36">
-        <v>4</v>
-      </c>
-      <c r="B16" s="35" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="36">
-        <v>5</v>
-      </c>
-      <c r="B17" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="36"/>
-      <c r="B18" s="35"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="36">
-        <v>6</v>
-      </c>
-      <c r="B19" s="35" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="36">
-        <v>7</v>
-      </c>
-      <c r="B20" s="44" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-    </row>
-    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
+      <c r="C31" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+    </row>
+    <row r="32" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="63"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="79"/>
+      <c r="D32" s="79"/>
+      <c r="E32" s="79"/>
+      <c r="F32" s="46"/>
+      <c r="G32" s="46"/>
+      <c r="H32" s="46"/>
+    </row>
+    <row r="33" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="45"/>
+      <c r="B33" s="53"/>
+      <c r="C33" s="80"/>
+      <c r="D33" s="81"/>
+      <c r="E33" s="81"/>
+      <c r="F33" s="51"/>
+      <c r="G33" s="51"/>
+      <c r="H33" s="52"/>
+    </row>
+    <row r="34" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="35" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="60" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C39" s="82"/>
+      <c r="D39" s="82"/>
+      <c r="E39" s="82"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Made changes to skip over non-docx templates in the clio_templates_sync.py script, added overrides for the --include-non-docx flag to allow for the inclusion of non-docx templates. Skipped over items are logged into replacement_report.csv.
</commit_message>
<xml_diff>
--- a/ClioCustomField_TestValidation.xlsx
+++ b/ClioCustomField_TestValidation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="685" documentId="8_{3120D6FD-25C6-47F0-8A39-89B25F99CA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A49D39BA-B205-48D6-87FC-457AC8C78DB6}"/>
+  <xr:revisionPtr revIDLastSave="843" documentId="8_{3120D6FD-25C6-47F0-8A39-89B25F99CA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47A6AC30-226F-49BD-A091-03DFFE7F3EBD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DF2C5E22-660C-4BCB-A765-9F1A84EF46AA}"/>
   </bookViews>
@@ -17,6 +17,9 @@
     <sheet name="EdgeTestingScenarios" sheetId="3" r:id="rId2"/>
     <sheet name="Templates" sheetId="2" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_Hlk108346204" localSheetId="1">EdgeTestingScenarios!$D$12</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="114">
   <si>
     <t>TempCode</t>
   </si>
@@ -184,9 +187,6 @@
     <t>&lt;&lt;Matter.CustomField.DefendantsFullLegalName &gt;&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;&lt;Matter.CustomField.Judge&gt;&gt; </t>
-  </si>
-  <si>
     <t>&lt;&lt; Matter.CustomField.County &gt;&gt;</t>
   </si>
   <si>
@@ -237,9 +237,6 @@
     </r>
   </si>
   <si>
-    <t>MCS Custom Field 2: 3 Spaces on Beginning of CF (split between pages,  7 CFs Within Template)</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <i/>
@@ -463,24 +460,9 @@
     <t>Mixed Case / Spacing in Custom Fields - Negative Testing</t>
   </si>
   <si>
-    <t>Custom Fields in Templates</t>
-  </si>
-  <si>
-    <t>Custom Fields in Lookup Tables</t>
-  </si>
-  <si>
     <t>Uppercase/Lower Case Testing Scenario does not follow the Positive/Negative Testing Basis</t>
   </si>
   <si>
-    <t>&lt;&lt; Matter.CustomField.CaseNumber &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.DefendantsFullLegalName &gt;&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;&lt; Matter.CustomField.Judge &gt;&gt; </t>
-  </si>
-  <si>
     <t>No Custom Field</t>
   </si>
   <si>
@@ -499,7 +481,236 @@
     <t>Custom Fields are Successfully Updated within each testing scenarios table, headers, and footers CF location</t>
   </si>
   <si>
+    <t>&lt;&lt;Matter.CustomField.CaseNumber &gt;&gt;</t>
+  </si>
+  <si>
     <t>&lt;&lt; MATTER.RESPONSIBLEATTORNEY.EMAIL &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.ResponsibleAttorney_Change3SpaceEndCF   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   MATTER.CUSTOMFIELD.PLAINTIFFSNAMESHORT_Change3SpaceBegCF &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.PlaintiffsFullLegalName_Change3SpaceEndBegCF   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CaseNumber_ChangeNoSpaceEndCF&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.DefendantsFullLegalName_ChangeNoSpaceBegCF &gt;&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;&lt;Matter.CustomField.Judge_ChangeNoSpaceEndBegCF&gt;&gt; </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">MCS Custom Field 2: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3 Spaces on Beginning of CF (split between pages,  6 Original CFs Within Template, 1 Test CF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">MCS Custom Field 3: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3 Spaces on Both Beg. and End of CF (2 Original CFs Within Template, 1 Test CF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 4:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No Spaces on End of CF (2 Original CFs Within Template. 1 Test CF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 5:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> No Spaces on Beg. of CF (2 Original CFs Within Template. 1 Test CF)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 6:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> No Spaces on Both Beg. And End of CF (2 Original CFs Within Template. 1 Test CF)</t>
+    </r>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.Judge&gt;&gt;</t>
+  </si>
+  <si>
+    <t>Old Custom Fields in Templates</t>
+  </si>
+  <si>
+    <t>New Custom Fields in Lookup Tables</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MCS Custom Field 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: 3 Spaces on End of CF </t>
+    </r>
+  </si>
+  <si>
+    <t>&lt;&lt; Date.Verbose   &gt;&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCS Custom Field 2: 3 Spaces on Beginning of CF </t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.CaseNameLong &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.OcStreetAddress   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney.email &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OcCityStateZip&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.CaseNameLong&gt;&gt;</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>Purposeply Slightly Incorrect CF Values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used to Validate Neg. Testing - If Below Values are Found Neg. Test Unsuccessfull </t>
+  </si>
+  <si>
+    <t>&lt;&lt; Date.Verbose_Change1&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.CaseNameLong_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;   Matter.CustomField.OcStreetAddress_Change1   &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OcCityStateZip_Change1&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.CaseNumber_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.CaseNameLong_Change1&gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney.email_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Success </t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.County_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OcCityStateZip_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OcStreetAddress_Change1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>Nothing Happens</t>
+  </si>
+  <si>
+    <t>Script downloaded the Excel File as a .docx (unable to open) when running Script to Update for an Error --&gt; Need to edit script to either only download .docx files, because we created a corrupted file even if we tried to skip over Update Script trying to then skip over Upload Script is just too much hassel. Final conclusion need to restrict to only download .docx files.</t>
   </si>
 </sst>
 </file>
@@ -509,7 +720,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="."/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -560,8 +771,17 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -652,8 +872,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8F8F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="21">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -913,11 +1151,54 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1011,17 +1292,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1071,9 +1346,6 @@
     <xf numFmtId="164" fontId="6" fillId="14" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1083,6 +1355,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1114,6 +1389,63 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1154,6 +1486,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF8F8F"/>
       <color rgb="FFFFFF99"/>
     </mruColors>
   </colors>
@@ -1737,553 +2070,604 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="88.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.42578125" style="40" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.42578125" style="40" customWidth="1"/>
-    <col min="5" max="5" width="58.85546875" style="40" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="70.28515625" customWidth="1"/>
+    <col min="3" max="3" width="58.85546875" style="39" customWidth="1"/>
+    <col min="4" max="4" width="53.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="74.140625" style="39" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="48.5703125" customWidth="1"/>
-    <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="39.85546875" customWidth="1"/>
+    <col min="7" max="7" width="51.7109375" customWidth="1"/>
+    <col min="8" max="8" width="94.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="40" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57"/>
-      <c r="B1" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="C1" s="39" t="s">
-        <v>69</v>
-      </c>
-      <c r="D1" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="E1" s="39" t="s">
-        <v>56</v>
-      </c>
-      <c r="F1" s="39" t="s">
-        <v>62</v>
-      </c>
-      <c r="G1" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="H1" s="39" t="s">
+    <row r="1" spans="1:8" s="39" customFormat="1" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="55"/>
+      <c r="B1" s="83" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="84" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="84" t="s">
+        <v>88</v>
+      </c>
+      <c r="E1" s="84" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="84" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="84" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="84" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="59"/>
+      <c r="B2" s="52" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="54"/>
+    </row>
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="60"/>
+      <c r="B3" s="85" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="61"/>
-      <c r="B2" s="54" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="56"/>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="62"/>
-      <c r="B3" s="36" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="86" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="94" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="77" t="s">
-        <v>59</v>
-      </c>
-      <c r="F3" s="67"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="33"/>
-    </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="62"/>
+      <c r="E3" s="87" t="s">
+        <v>76</v>
+      </c>
+      <c r="F3" s="64"/>
+      <c r="G3" s="88" t="s">
+        <v>98</v>
+      </c>
+      <c r="H3" s="88"/>
+    </row>
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="60"/>
       <c r="B4" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>31</v>
+        <v>82</v>
+      </c>
+      <c r="C4" s="75" t="s">
+        <v>57</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="77" t="s">
-        <v>59</v>
-      </c>
-      <c r="F4" s="68"/>
-      <c r="G4" s="65"/>
+      <c r="E4" s="82" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" s="65"/>
+      <c r="G4" s="33" t="s">
+        <v>98</v>
+      </c>
       <c r="H4" s="33"/>
     </row>
-    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="62"/>
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="60"/>
       <c r="B5" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" s="75" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="77" t="s">
-        <v>59</v>
-      </c>
-      <c r="F5" s="68"/>
-      <c r="G5" s="65"/>
+      <c r="E5" s="81" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" s="65"/>
+      <c r="G5" s="33" t="s">
+        <v>98</v>
+      </c>
       <c r="H5" s="33"/>
     </row>
     <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="62">
+      <c r="A6" s="60">
         <v>1</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>34</v>
+        <v>84</v>
+      </c>
+      <c r="C6" s="75" t="s">
+        <v>57</v>
       </c>
       <c r="D6" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="77" t="s">
-        <v>59</v>
-      </c>
-      <c r="F6" s="70" t="s">
-        <v>78</v>
-      </c>
-      <c r="G6" s="65"/>
+      <c r="E6" s="82" t="s">
+        <v>79</v>
+      </c>
+      <c r="F6" s="68" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="33" t="s">
+        <v>98</v>
+      </c>
       <c r="H6" s="33"/>
     </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="62"/>
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="60"/>
       <c r="B7" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7" s="75" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="95" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="81" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" s="65"/>
+      <c r="G7" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="H7" s="33"/>
+    </row>
+    <row r="8" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="60"/>
+      <c r="B8" s="92" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" s="91" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="89" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" s="93" t="s">
+        <v>81</v>
+      </c>
+      <c r="F8" s="66"/>
+      <c r="G8" s="90" t="s">
+        <v>98</v>
+      </c>
+      <c r="H8" s="90"/>
+    </row>
+    <row r="9" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="60"/>
+      <c r="B9" s="57" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="75" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="81" t="s">
+        <v>95</v>
+      </c>
+      <c r="E9" s="81" t="s">
+        <v>107</v>
+      </c>
+      <c r="F9" s="66"/>
+      <c r="G9" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="H9" s="33"/>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="61"/>
+      <c r="B10" s="42"/>
+      <c r="C10" s="89"/>
+      <c r="D10" s="89"/>
+      <c r="E10" s="89"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43"/>
+      <c r="H10" s="43"/>
+    </row>
+    <row r="11" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="59"/>
+      <c r="B11" s="52" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="74"/>
+      <c r="D11" s="96" t="s">
+        <v>99</v>
+      </c>
+      <c r="E11" s="96" t="s">
+        <v>100</v>
+      </c>
+      <c r="F11" s="53"/>
+      <c r="G11" s="53"/>
+      <c r="H11" s="54"/>
+    </row>
+    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="60"/>
+      <c r="B12" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="81" t="s">
+        <v>91</v>
+      </c>
+      <c r="E12" s="81" t="s">
+        <v>101</v>
+      </c>
+      <c r="F12" s="67"/>
+      <c r="G12" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="H12" s="33"/>
+    </row>
+    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="60"/>
+      <c r="B13" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="82" t="s">
+        <v>93</v>
+      </c>
+      <c r="E13" s="82" t="s">
+        <v>102</v>
+      </c>
+      <c r="F13" s="65"/>
+      <c r="G13" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="H13" s="33"/>
+    </row>
+    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="60"/>
+      <c r="B14" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="81" t="s">
+        <v>94</v>
+      </c>
+      <c r="E14" s="81" t="s">
+        <v>103</v>
+      </c>
+      <c r="F14" s="65"/>
+      <c r="G14" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="H14" s="33"/>
+    </row>
+    <row r="15" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="60">
+        <v>2</v>
+      </c>
+      <c r="B15" s="36" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="82" t="s">
+        <v>96</v>
+      </c>
+      <c r="E15" s="82" t="s">
+        <v>104</v>
+      </c>
+      <c r="F15" s="68" t="s">
+        <v>72</v>
+      </c>
+      <c r="G15" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="H15" s="33"/>
+    </row>
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="60"/>
+      <c r="B16" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="81" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16" s="81" t="s">
+        <v>105</v>
+      </c>
+      <c r="F16" s="65"/>
+      <c r="G16" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="H16" s="33"/>
+    </row>
+    <row r="17" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="60"/>
+      <c r="B17" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="82" t="s">
+        <v>97</v>
+      </c>
+      <c r="E17" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="F17" s="65"/>
+      <c r="G17" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="H17" s="33"/>
+    </row>
+    <row r="18" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="61"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="76"/>
+      <c r="D18" s="76"/>
+      <c r="E18" s="76"/>
+      <c r="F18" s="69"/>
+      <c r="G18" s="48"/>
+      <c r="H18" s="48"/>
+    </row>
+    <row r="19" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="59"/>
+      <c r="B19" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" s="74"/>
+      <c r="D19" s="74"/>
+      <c r="E19" s="74"/>
+      <c r="F19" s="63"/>
+      <c r="G19" s="53"/>
+      <c r="H19" s="54"/>
+    </row>
+    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="60"/>
+      <c r="B20" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="77" t="s">
-        <v>59</v>
-      </c>
-      <c r="F7" s="68"/>
-      <c r="G7" s="65"/>
-      <c r="H7" s="33"/>
-    </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="62"/>
-      <c r="B8" s="36" t="s">
+      <c r="C20" s="75" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="81" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="81" t="s">
+        <v>109</v>
+      </c>
+      <c r="F20" s="71"/>
+      <c r="G20" s="70" t="s">
+        <v>98</v>
+      </c>
+      <c r="H20" s="22"/>
+    </row>
+    <row r="21" spans="1:8" s="39" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A21" s="56">
+        <v>3</v>
+      </c>
+      <c r="B21" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="E8" s="77" t="s">
-        <v>59</v>
-      </c>
-      <c r="F8" s="68"/>
-      <c r="G8" s="65"/>
-      <c r="H8" s="33"/>
-    </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="62"/>
-      <c r="B9" s="59" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" s="77" t="s">
+      <c r="C21" s="73" t="s">
         <v>58</v>
       </c>
-      <c r="F9" s="69"/>
-      <c r="G9" s="65"/>
-      <c r="H9" s="33"/>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="63"/>
-      <c r="B10" s="44"/>
-      <c r="C10" s="78"/>
-      <c r="D10" s="78"/>
-      <c r="E10" s="78"/>
-      <c r="F10" s="50"/>
-      <c r="G10" s="50"/>
-      <c r="H10" s="50"/>
-    </row>
-    <row r="11" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="61"/>
-      <c r="B11" s="54" t="s">
+      <c r="D21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F21" s="68" t="s">
+        <v>73</v>
+      </c>
+      <c r="G21" s="98" t="s">
+        <v>98</v>
+      </c>
+      <c r="H21" s="1"/>
+    </row>
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="60"/>
+      <c r="B22" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="73" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" s="97" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" s="97" t="s">
+        <v>111</v>
+      </c>
+      <c r="F22" s="72"/>
+      <c r="G22" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="H22" s="3"/>
+    </row>
+    <row r="23" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="61"/>
+      <c r="B23" s="45"/>
+      <c r="C23" s="77"/>
+      <c r="D23" s="77"/>
+      <c r="E23" s="77"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="44"/>
+    </row>
+    <row r="24" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="59"/>
+      <c r="B24" s="52" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="74"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="74"/>
+      <c r="F24" s="53"/>
+      <c r="G24" s="53"/>
+      <c r="H24" s="54"/>
+    </row>
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="60"/>
+      <c r="B25" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="C11" s="76"/>
-      <c r="D11" s="76"/>
-      <c r="E11" s="76"/>
-      <c r="F11" s="55"/>
-      <c r="G11" s="55"/>
-      <c r="H11" s="56"/>
-    </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="62"/>
-      <c r="B12" s="36" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="F12" s="67"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="33"/>
-    </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="62"/>
-      <c r="B13" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="F13" s="68"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="33"/>
-    </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="62"/>
-      <c r="B14" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="F14" s="68"/>
-      <c r="G14" s="33"/>
-      <c r="H14" s="33"/>
-    </row>
-    <row r="15" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="62">
-        <v>2</v>
-      </c>
-      <c r="B15" s="36" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="E15" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="F15" s="70" t="s">
-        <v>79</v>
-      </c>
-      <c r="G15" s="33"/>
-      <c r="H15" s="33"/>
-    </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="62"/>
-      <c r="B16" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="E16" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="F16" s="68"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="33"/>
-    </row>
-    <row r="17" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="62"/>
-      <c r="B17" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="E17" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="F17" s="68"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="33"/>
-    </row>
-    <row r="18" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="63"/>
-      <c r="B18" s="44"/>
-      <c r="C18" s="78"/>
-      <c r="D18" s="78"/>
-      <c r="E18" s="78"/>
-      <c r="F18" s="71"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
-    </row>
-    <row r="19" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="61"/>
-      <c r="B19" s="54" t="s">
-        <v>64</v>
-      </c>
-      <c r="C19" s="76"/>
-      <c r="D19" s="76"/>
-      <c r="E19" s="76"/>
-      <c r="F19" s="66"/>
-      <c r="G19" s="55"/>
-      <c r="H19" s="56"/>
-    </row>
-    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="62"/>
-      <c r="B20" s="48" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="E20" s="77" t="s">
-        <v>60</v>
-      </c>
-      <c r="F20" s="73"/>
-      <c r="G20" s="72"/>
-      <c r="H20" s="22"/>
-    </row>
-    <row r="21" spans="1:8" s="40" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="58">
-        <v>3</v>
-      </c>
-      <c r="B21" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E21" s="75" t="s">
-        <v>60</v>
-      </c>
-      <c r="F21" s="70" t="s">
-        <v>80</v>
-      </c>
-      <c r="G21" s="10"/>
-      <c r="H21" s="1"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="62"/>
-      <c r="B22" s="35" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E22" s="75" t="s">
-        <v>60</v>
-      </c>
-      <c r="F22" s="74"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="3"/>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="63"/>
-      <c r="B23" s="47"/>
-      <c r="C23" s="79"/>
-      <c r="D23" s="79"/>
-      <c r="E23" s="79"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="46"/>
-      <c r="H23" s="46"/>
-    </row>
-    <row r="24" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="61"/>
-      <c r="B24" s="54" t="s">
-        <v>65</v>
-      </c>
-      <c r="C24" s="76"/>
-      <c r="D24" s="76"/>
-      <c r="E24" s="76"/>
-      <c r="F24" s="55"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="56"/>
-    </row>
-    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="62"/>
-      <c r="B25" s="49" t="s">
-        <v>26</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="E25" s="20"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
+      <c r="F25" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="G25" s="22" t="s">
+        <v>98</v>
+      </c>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="62">
+    <row r="26" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="60">
         <v>4</v>
       </c>
       <c r="B26" s="34" t="s">
         <v>28</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
+      <c r="H26" s="99" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="62"/>
+      <c r="A27" s="60"/>
       <c r="B27" s="34" t="s">
         <v>29</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="63"/>
-      <c r="B28" s="41"/>
-      <c r="C28" s="79"/>
-      <c r="D28" s="79"/>
-      <c r="E28" s="79"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="46"/>
-      <c r="H28" s="46"/>
+      <c r="A28" s="61"/>
+      <c r="B28" s="40"/>
+      <c r="C28" s="77"/>
+      <c r="D28" s="77"/>
+      <c r="E28" s="77"/>
+      <c r="F28" s="44"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="44"/>
     </row>
     <row r="29" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="64"/>
-      <c r="B29" s="54" t="s">
-        <v>66</v>
-      </c>
-      <c r="C29" s="76"/>
-      <c r="D29" s="76"/>
-      <c r="E29" s="76"/>
-      <c r="F29" s="55"/>
-      <c r="G29" s="55"/>
-      <c r="H29" s="56"/>
+      <c r="A29" s="62"/>
+      <c r="B29" s="52" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" s="74"/>
+      <c r="D29" s="74"/>
+      <c r="E29" s="74"/>
+      <c r="F29" s="53"/>
+      <c r="G29" s="53"/>
+      <c r="H29" s="54"/>
     </row>
     <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="62"/>
-      <c r="B30" s="43" t="s">
+      <c r="A30" s="60"/>
+      <c r="B30" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="D30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20" t="s">
+        <v>43</v>
+      </c>
       <c r="E30" s="20"/>
       <c r="F30" s="22"/>
       <c r="G30" s="22"/>
       <c r="H30" s="22"/>
     </row>
     <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="62">
+      <c r="A31" s="60">
         <v>5</v>
       </c>
       <c r="B31" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="E31" s="1"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="63"/>
+      <c r="A32" s="61"/>
       <c r="B32" s="5"/>
-      <c r="C32" s="79"/>
-      <c r="D32" s="79"/>
-      <c r="E32" s="79"/>
-      <c r="F32" s="46"/>
-      <c r="G32" s="46"/>
-      <c r="H32" s="46"/>
+      <c r="C32" s="77"/>
+      <c r="D32" s="77"/>
+      <c r="E32" s="77"/>
+      <c r="F32" s="44"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="44"/>
     </row>
     <row r="33" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="45"/>
-      <c r="B33" s="53"/>
-      <c r="C33" s="80"/>
-      <c r="D33" s="81"/>
-      <c r="E33" s="81"/>
-      <c r="F33" s="51"/>
-      <c r="G33" s="51"/>
-      <c r="H33" s="52"/>
+      <c r="A33" s="43"/>
+      <c r="B33" s="51"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="78"/>
+      <c r="E33" s="79"/>
+      <c r="F33" s="49"/>
+      <c r="G33" s="49"/>
+      <c r="H33" s="50"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="35" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="60" t="s">
-        <v>71</v>
+      <c r="B35" s="58" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D36" s="39" t="s">
+        <v>75</v>
+      </c>
+      <c r="E36" s="39" t="str">
+        <f>LOWER(D36)</f>
+        <v>&lt;&lt; matter.responsibleattorney.email &gt;&gt;</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C39" s="82"/>
-      <c r="D39" s="82"/>
-      <c r="E39" s="82"/>
+      <c r="C39" s="80"/>
+      <c r="D39" s="80"/>
+      <c r="E39" s="80"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>